<commit_message>
chore(bugs): back-fill TS-* Fix Commit cells with SHA b77e1a4
Replaces the "(pending — this commit)" placeholder in the 36 TS-*
Fix Commit cells with the actual commit SHA of the parent fix-batch
(b77e1a4 "fix(bugs): close 36 Open TS-* test-scenarios-xlsx
meta-bugs").

Same back-fill pattern that bbea337 used for the legacy BUG-NNN
entries via populate_bug_fix_commits_2026_05_17.py. The current
populate tool is BUG-NNN-only; this back-fill is a one-shot manual
edit (36 cells updated) rather than extending the tool — TS-* are
a finite class produced by a single audit pass, unlike BUG-NNN
which is open-ended.

JA-118 (every Fixed row has non-empty Fix Commit) PASSed with the
placeholder; passes again with the SHA. Update is informational +
back-links to the canonical fix commit for future audit traceability.

Final bug-tracker state: 89 / 89 Fixed / 0 Open.
CI: 122/122 invariants green.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/N5/specifications/test-scenarios-by-specialist-perspective.xlsx
+++ b/N5/specifications/test-scenarios-by-specialist-perspective.xlsx
@@ -23464,7 +23464,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N57" s="58" t="n">
@@ -23520,7 +23520,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N58" s="58" t="n">
@@ -23573,7 +23573,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N59" s="58" t="n">
@@ -23629,7 +23629,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N60" s="58" t="n">
@@ -23685,7 +23685,7 @@
       </c>
       <c r="M61" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N61" s="58" t="n">
@@ -23743,7 +23743,7 @@
       </c>
       <c r="M62" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N62" s="58" t="n">
@@ -23799,7 +23799,7 @@
       </c>
       <c r="M63" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N63" s="58" t="n">
@@ -23860,7 +23860,7 @@
       </c>
       <c r="M64" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N64" s="58" t="n">
@@ -23921,7 +23921,7 @@
       </c>
       <c r="M65" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N65" s="58" t="n">
@@ -23976,7 +23976,7 @@
       </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N66" s="58" t="n">
@@ -24029,7 +24029,7 @@
       </c>
       <c r="M67" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N67" s="58" t="n">
@@ -24088,7 +24088,7 @@
       </c>
       <c r="M68" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N68" s="58" t="n">
@@ -24144,7 +24144,7 @@
       </c>
       <c r="M69" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N69" s="58" t="n">
@@ -24199,7 +24199,7 @@
       </c>
       <c r="M70" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N70" s="58" t="n">
@@ -24255,7 +24255,7 @@
       </c>
       <c r="M71" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N71" s="58" t="n">
@@ -24315,7 +24315,7 @@
       </c>
       <c r="M72" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N72" s="58" t="n">
@@ -24370,7 +24370,7 @@
       </c>
       <c r="M73" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N73" s="58" t="n">
@@ -24428,7 +24428,7 @@
       </c>
       <c r="M74" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N74" s="58" t="n">
@@ -24488,7 +24488,7 @@
       </c>
       <c r="M75" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N75" s="58" t="n">
@@ -24551,7 +24551,7 @@
       </c>
       <c r="M76" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N76" s="58" t="n">
@@ -24610,7 +24610,7 @@
       </c>
       <c r="M77" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N77" s="58" t="n">
@@ -24666,7 +24666,7 @@
       </c>
       <c r="M78" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N78" s="58" t="n">
@@ -24720,7 +24720,7 @@
       </c>
       <c r="M79" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N79" s="58" t="n">
@@ -24773,7 +24773,7 @@
       </c>
       <c r="M80" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N80" s="58" t="n">
@@ -24830,7 +24830,7 @@
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N81" s="58" t="n">
@@ -24884,7 +24884,7 @@
       </c>
       <c r="M82" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N82" s="58" t="n">
@@ -24940,7 +24940,7 @@
       </c>
       <c r="M83" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N83" s="58" t="n">
@@ -24995,7 +24995,7 @@
       </c>
       <c r="M84" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N84" s="58" t="n">
@@ -25051,7 +25051,7 @@
       </c>
       <c r="M85" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N85" s="58" t="n">
@@ -25106,7 +25106,7 @@
       </c>
       <c r="M86" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N86" s="58" t="n">
@@ -25160,7 +25160,7 @@
       </c>
       <c r="M87" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N87" s="58" t="n">
@@ -25216,7 +25216,7 @@
       </c>
       <c r="M88" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N88" s="58" t="n">
@@ -25273,7 +25273,7 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N89" s="58" t="n">
@@ -25326,7 +25326,7 @@
       </c>
       <c r="M90" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N90" s="58" t="n">
@@ -25382,7 +25382,7 @@
       </c>
       <c r="M91" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N91" s="58" t="n">
@@ -25443,7 +25443,7 @@
       </c>
       <c r="M92" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>b77e1a4</t>
         </is>
       </c>
       <c r="N92" s="58" t="n">

</xml_diff>

<commit_message>
chore(bugs): migrate NR-* Fix Commit cells to col 9 + backfill SHA d26e677
The original bug-filer wrote Fix Commit + Fix Date to cols 13/14
(stale schema position based on a pre-fix_ts_bugs xlsx state); the
current xlsx layout has those fields at cols 9/10. Migrated 5 NR-*
rows accordingly. JA-118 PASS (94/94 Fixed rows have non-empty
Fix Commit cell).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/N5/specifications/test-scenarios-by-specialist-perspective.xlsx
+++ b/N5/specifications/test-scenarios-by-specialist-perspective.xlsx
@@ -25995,14 +25995,15 @@
           <t>Fixed</t>
         </is>
       </c>
-      <c r="M93" t="inlineStr">
-        <is>
-          <t>(pending — this commit)</t>
-        </is>
-      </c>
-      <c r="N93" s="68" t="n">
-        <v>46159</v>
-      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>d26e677</t>
+        </is>
+      </c>
+      <c r="J93" s="68" t="n">
+        <v>46159</v>
+      </c>
+      <c r="N93" s="68" t="n"/>
     </row>
     <row r="94">
       <c r="B94" s="2" t="n">
@@ -26040,14 +26041,15 @@
           <t>Fixed</t>
         </is>
       </c>
-      <c r="M94" t="inlineStr">
-        <is>
-          <t>(pending — this commit)</t>
-        </is>
-      </c>
-      <c r="N94" s="68" t="n">
-        <v>46159</v>
-      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>d26e677</t>
+        </is>
+      </c>
+      <c r="J94" s="68" t="n">
+        <v>46159</v>
+      </c>
+      <c r="N94" s="68" t="n"/>
     </row>
     <row r="95">
       <c r="B95" s="2" t="n">
@@ -26086,14 +26088,15 @@
           <t>Fixed</t>
         </is>
       </c>
-      <c r="M95" t="inlineStr">
-        <is>
-          <t>(pending — this commit)</t>
-        </is>
-      </c>
-      <c r="N95" s="68" t="n">
-        <v>46159</v>
-      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>d26e677</t>
+        </is>
+      </c>
+      <c r="J95" s="68" t="n">
+        <v>46159</v>
+      </c>
+      <c r="N95" s="68" t="n"/>
     </row>
     <row r="96">
       <c r="B96" s="2" t="n">
@@ -26132,14 +26135,15 @@
           <t>Fixed</t>
         </is>
       </c>
-      <c r="M96" t="inlineStr">
-        <is>
-          <t>(pending — this commit)</t>
-        </is>
-      </c>
-      <c r="N96" s="68" t="n">
-        <v>46159</v>
-      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>d26e677</t>
+        </is>
+      </c>
+      <c r="J96" s="68" t="n">
+        <v>46159</v>
+      </c>
+      <c r="N96" s="68" t="n"/>
     </row>
     <row r="97">
       <c r="B97" s="2" t="n">
@@ -26193,14 +26197,15 @@
           <t>Fixed</t>
         </is>
       </c>
-      <c r="M97" t="inlineStr">
-        <is>
-          <t>(pending — this commit)</t>
-        </is>
-      </c>
-      <c r="N97" s="68" t="n">
-        <v>46159</v>
-      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>d26e677</t>
+        </is>
+      </c>
+      <c r="J97" s="68" t="n">
+        <v>46159</v>
+      </c>
+      <c r="N97" s="68" t="n"/>
     </row>
     <row r="98">
       <c r="B98" s="2" t="n"/>

</xml_diff>

<commit_message>
chore(bugs): back-fill NR-HI/NR-JE Fix Commit cells with 8159b49
</commit_message>
<xml_diff>
--- a/N5/specifications/test-scenarios-by-specialist-perspective.xlsx
+++ b/N5/specifications/test-scenarios-by-specialist-perspective.xlsx
@@ -26246,7 +26246,7 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>8159b49</t>
         </is>
       </c>
       <c r="J98" s="68" t="n">
@@ -26292,7 +26292,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>8159b49</t>
         </is>
       </c>
       <c r="J99" s="68" t="n">
@@ -26338,7 +26338,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>8159b49</t>
         </is>
       </c>
       <c r="J100" s="68" t="n">
@@ -26389,7 +26389,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>8159b49</t>
         </is>
       </c>
       <c r="J101" s="68" t="n">

</xml_diff>

<commit_message>
chore(bugs): back-fill NR-SEC/LIC/DATA Fix Commit cells with 46be3e1
</commit_message>
<xml_diff>
--- a/N5/specifications/test-scenarios-by-specialist-perspective.xlsx
+++ b/N5/specifications/test-scenarios-by-specialist-perspective.xlsx
@@ -26435,7 +26435,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>46be3e1</t>
         </is>
       </c>
       <c r="J102" s="68" t="n">
@@ -26488,7 +26488,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>46be3e1</t>
         </is>
       </c>
       <c r="J103" s="68" t="n">
@@ -26534,7 +26534,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>46be3e1</t>
         </is>
       </c>
       <c r="J104" s="68" t="n">
@@ -26584,7 +26584,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>(pending — this commit)</t>
+          <t>46be3e1</t>
         </is>
       </c>
       <c r="J105" s="68" t="n">

</xml_diff>

<commit_message>
chore(bugs): back-fill BUG-050 / 090..093 Fix Commit with 7728348
Replaces the previous "(pending — this commit closes
PAPER-001..004 + LISTEN-4)" placeholder with the actual commit
hash from 7728348 (the PAPER-001..004 + LISTEN-4 close-out
commit).

Mechanical change only — no methodology implication. Skipped
doc updates per the BINDING Rule 4 mechanical-change exception.

JA-118 (every Fixed row has non-empty Fix Commit) continues to
PASS; this commit just upgrades the placeholder to the real
hash so the cell value is verifiable against `git log`.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/N5/specifications/test-scenarios-by-specialist-perspective.xlsx
+++ b/N5/specifications/test-scenarios-by-specialist-perspective.xlsx
@@ -24096,7 +24096,7 @@
       </c>
       <c r="I53" s="54" t="inlineStr">
         <is>
-          <t>(pending — this commit closes PAPER-001..004 + LISTEN-4)</t>
+          <t>7728348</t>
         </is>
       </c>
       <c r="J53" s="53" t="inlineStr">
@@ -26396,7 +26396,7 @@
       </c>
       <c r="I93" s="3" t="inlineStr">
         <is>
-          <t>(pending — this commit closes PAPER-001..004 + LISTEN-4)</t>
+          <t>7728348</t>
         </is>
       </c>
       <c r="J93" s="74" t="inlineStr">
@@ -26455,7 +26455,7 @@
       </c>
       <c r="I94" s="3" t="inlineStr">
         <is>
-          <t>(pending — this commit closes PAPER-001..004 + LISTEN-4)</t>
+          <t>7728348</t>
         </is>
       </c>
       <c r="J94" s="74" t="inlineStr">
@@ -26535,7 +26535,7 @@
       </c>
       <c r="I95" s="3" t="inlineStr">
         <is>
-          <t>(pending — this commit closes PAPER-001..004 + LISTEN-4)</t>
+          <t>7728348</t>
         </is>
       </c>
       <c r="J95" s="74" t="inlineStr">
@@ -26619,7 +26619,7 @@
       </c>
       <c r="I96" s="10" t="inlineStr">
         <is>
-          <t>(pending — this commit closes PAPER-001..004 + LISTEN-4)</t>
+          <t>7728348</t>
         </is>
       </c>
       <c r="J96" s="84" t="inlineStr">

</xml_diff>

<commit_message>
chore(bugs): back-fill BUG-094..097 / 105 / 106 Fix Commit with c55d7f6
Replaces the previous "(pending — this commit closes LLM-001..005 +
REG-001)" placeholder with the actual commit hash from c55d7f6 (the
LLM-001..005 + REG-001 close-out commit).

Mechanical change only — no methodology implication. Skipped doc
updates per the BINDING Rule 4 mechanical-change exception.

JA-118 (every Fixed row has non-empty Fix Commit) continues to PASS;
this commit just upgrades the placeholder to the real hash so the
cell value is verifiable against `git log`.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/N5/specifications/test-scenarios-by-specialist-perspective.xlsx
+++ b/N5/specifications/test-scenarios-by-specialist-perspective.xlsx
@@ -26788,7 +26788,7 @@
       </c>
       <c r="I97" s="86" t="inlineStr">
         <is>
-          <t>(pending — this commit closes LLM-001..005 + REG-001)</t>
+          <t>c55d7f6</t>
         </is>
       </c>
       <c r="J97" s="85" t="inlineStr">
@@ -26855,7 +26855,7 @@
       </c>
       <c r="I98" s="86" t="inlineStr">
         <is>
-          <t>(pending — this commit closes LLM-001..005 + REG-001)</t>
+          <t>c55d7f6</t>
         </is>
       </c>
       <c r="J98" s="85" t="inlineStr">
@@ -26922,7 +26922,7 @@
       </c>
       <c r="I99" s="86" t="inlineStr">
         <is>
-          <t>(pending — this commit closes LLM-001..005 + REG-001)</t>
+          <t>c55d7f6</t>
         </is>
       </c>
       <c r="J99" s="85" t="inlineStr">
@@ -27012,7 +27012,7 @@
       </c>
       <c r="I100" s="86" t="inlineStr">
         <is>
-          <t>(pending — this commit closes LLM-001..005 + REG-001)</t>
+          <t>c55d7f6</t>
         </is>
       </c>
       <c r="J100" s="85" t="inlineStr">
@@ -27486,7 +27486,7 @@
       </c>
       <c r="I108" s="87" t="inlineStr">
         <is>
-          <t>(pending — this commit closes LLM-001..005 + REG-001)</t>
+          <t>c55d7f6</t>
         </is>
       </c>
       <c r="J108" s="13" t="inlineStr">
@@ -27595,7 +27595,7 @@
       </c>
       <c r="I109" s="86" t="inlineStr">
         <is>
-          <t>(pending — this commit closes LLM-001..005 + REG-001)</t>
+          <t>c55d7f6</t>
         </is>
       </c>
       <c r="J109" s="88" t="inlineStr">

</xml_diff>